<commit_message>
Updated all template in editable form.
</commit_message>
<xml_diff>
--- a/FinanceDataMigration/src/main/resources/migration-templates/BANK.xlsx
+++ b/FinanceDataMigration/src/main/resources/migration-templates/BANK.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr/>
+  <workbookPr hidePivotFieldList="0"/>
   <bookViews>
     <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Bank " sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -28,9 +28,12 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <b/>
-        <color indexed="64"/>
+        <sz val="11"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">ULB Name </t>
@@ -38,6 +41,7 @@
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
         <color indexed="2"/>
         <rFont val="Arial"/>
       </rPr>
@@ -46,9 +50,12 @@
   </si>
   <si>
     <r>
+      <t/>
+    </r>
+    <r>
       <rPr>
         <b/>
-        <color indexed="64"/>
+        <sz val="11"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">Bank Name </t>
@@ -56,6 +63,7 @@
     <r>
       <rPr>
         <b/>
+        <sz val="11"/>
         <color indexed="2"/>
         <rFont val="Arial"/>
       </rPr>
@@ -213,31 +221,27 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="5">
     <font>
-      <sz val="11.000000"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
+      <sz val="10.000000"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="11.000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <color rgb="FFC9211E"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
       <color indexed="64"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <color rgb="FFC9211E"/>
+      <sz val="11.000000"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <color indexed="64"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -250,37 +254,28 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF6FA8DC"/>
-        <bgColor rgb="FF6FA8DC"/>
+        <bgColor indexed="55"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEAD1DC"/>
-        <bgColor rgb="FFEAD1DC"/>
+        <bgColor indexed="47"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFB6D7A8"/>
-        <bgColor rgb="FFB6D7A8"/>
+        <bgColor rgb="FFEAD1DC"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left style="none"/>
       <right style="none"/>
       <top style="none"/>
       <bottom style="none"/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal style="none"/>
     </border>
     <border>
@@ -299,8 +294,13 @@
       <diagonal style="none"/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="43" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="41" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="44" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
@@ -310,28 +310,30 @@
     <xf fontId="2" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="1" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="1" fillId="4" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="4" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="4" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
+    <cellStyle name="Currency" xfId="3" builtinId="4"/>
+    <cellStyle name="Currency[0]" xfId="4" builtinId="7"/>
+    <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -621,49 +623,49 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="">
   <a:themeElements>
-    <a:clrScheme name="New Office">
+    <a:clrScheme name="">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface="Arial"/>
         <a:cs typeface="Arial"/>
       </a:majorFont>
@@ -673,7 +675,7 @@
         <a:cs typeface="Arial"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -682,76 +684,67 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+        <a:ln w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -776,38 +769,11 @@
           <a:schemeClr val="phClr"/>
         </a:solidFill>
         <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
+          <a:srgbClr val="000000"/>
         </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
@@ -817,7 +783,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetPr>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="12.800000000000001" customHeight="1"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="11.5352"/>
+    <col customWidth="1" min="2" max="2" width="28.109400000000001"/>
+    <col customWidth="1" min="3" max="3" width="39.039099999999998"/>
+    <col customWidth="1" min="4" max="4" width="26.921900000000001"/>
+    <col customWidth="1" min="5" max="257" width="11.5352"/>
+  </cols>
   <sheetData>
     <row r="1" ht="14.25">
       <c r="A1" s="1" t="s">
@@ -1400,6 +1377,12 @@
         <v>52</v>
       </c>
       <c r="D49" s="5"/>
+    </row>
+    <row r="50" ht="14.25">
+      <c r="A50" s="5"/>
+      <c r="B50" s="5"/>
+      <c r="C50" s="5"/>
+      <c r="D50" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1407,25 +1390,14 @@
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <dataValidations count="1" disablePrompts="0">
-    <dataValidation sqref="B4:B49" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="0">
-      <formula1>'DropDown List'!$A$2:$A$1000</formula1>
-    </dataValidation>
+    <dataValidation sqref="1:1048576" type="none" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1"/>
   </dataValidations>
   <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="0" copies="1"/>
-  <headerFooter/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{A0E49462-1D10-4F78-833E-4DECA01E7CE4}" type="custom" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="1" showErrorMessage="1" showInputMessage="0">
-          <x14:formula1>
-            <xm:f>COUNTIF($C$4:$C$1000,C4)=1</xm:f>
-          </x14:formula1>
-          <xm:sqref>C4:C49</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
+  <pageMargins left="0.78750000000000009" right="0.78750000000000009" top="1.052778" bottom="1.052778" header="0.78750000000000009" footer="0.78750000000000009"/>
+  <pageSetup paperSize="9" scale="90" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>